<commit_message>
corrected the bulk search
</commit_message>
<xml_diff>
--- a/bulk-results/results_1.xlsx
+++ b/bulk-results/results_1.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O24"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="35.83203125" customWidth="1"/>
@@ -501,13 +501,13 @@
         <v>100 000 DHS</v>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>N°00-62 lot al massira - Ouarzazate (M)</v>
       </c>
       <c r="N2" t="str">
         <v/>
       </c>
       <c r="O2">
-        <v>5065</v>
+        <v>8944</v>
       </c>
     </row>
     <row r="3">
@@ -548,13 +548,13 @@
         <v>100 000 DHS</v>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>Lotissement el afaq n° 1048 - Marrakech-Médina (AR)</v>
       </c>
       <c r="N3" t="str">
         <v/>
       </c>
       <c r="O3">
-        <v>3032</v>
+        <v>24762</v>
       </c>
     </row>
     <row r="4">
@@ -595,13 +595,13 @@
         <v>500 000 DHS</v>
       </c>
       <c r="M4" t="str">
-        <v/>
+        <v>Rue bajjou douar bajjou cr iaazanen - Iaazzanene</v>
       </c>
       <c r="N4" t="str">
         <v/>
       </c>
       <c r="O4">
-        <v>2969</v>
+        <v>6956</v>
       </c>
     </row>
     <row r="5">
@@ -642,13 +642,13 @@
         <v>100 000 DHS</v>
       </c>
       <c r="M5" t="str">
-        <v/>
+        <v>Lot agdal n°404 bis 14200 - Sidi Slimane (M)</v>
       </c>
       <c r="N5" t="str">
         <v/>
       </c>
       <c r="O5">
-        <v>1813</v>
+        <v>11745</v>
       </c>
     </row>
     <row r="6">
@@ -689,13 +689,13 @@
         <v>100 000 DHS</v>
       </c>
       <c r="M6" t="str">
-        <v/>
+        <v>14, 2éme étage appt n° 03 bloc d hay essalam 14200 - Sidi Slimane (M)</v>
       </c>
       <c r="N6" t="str">
         <v/>
       </c>
       <c r="O6">
-        <v>1737</v>
+        <v>11625</v>
       </c>
     </row>
     <row r="7">
@@ -712,19 +712,19 @@
         <v>Not Found – Suggestion</v>
       </c>
       <c r="E7" t="str">
-        <v>STE TRAVAUX DE CONSTRUCTION MAHDID (SOTRACOMA)</v>
+        <v>SITANOR</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="str">
-        <v>21.7%</v>
+        <v>85.7%</v>
       </c>
       <c r="H7" t="str">
-        <v/>
+        <v>000050977000051</v>
       </c>
       <c r="I7" t="str">
-        <v>16611</v>
+        <v>22121</v>
       </c>
       <c r="J7" t="str">
         <v>Tribunal de Oujda</v>
@@ -733,16 +733,16 @@
         <v>Société à Responsabilité Limitée à Associé Unique</v>
       </c>
       <c r="L7" t="str">
-        <v>100 000 DHS</v>
+        <v>10 000 DHS</v>
       </c>
       <c r="M7" t="str">
-        <v>12 rue a 3 lot benkhirane route aouaja - Oujda (M)</v>
+        <v>3ème étage bd zerktouni residence zerktouni - Oujda (M)</v>
       </c>
       <c r="N7" t="str">
         <v/>
       </c>
       <c r="O7">
-        <v>3599</v>
+        <v>62438</v>
       </c>
     </row>
     <row r="8">
@@ -759,22 +759,22 @@
         <v>Not Found – Suggestion</v>
       </c>
       <c r="E8" t="str">
-        <v>SOCIETE MAROCAINE DE CONSTRUCTION ET DU DEVELOPPEMENT URBAIN ET RURAL "SARL" (STE SCOMADEUR SARL)</v>
+        <v>SOCANOR</v>
       </c>
       <c r="F8">
         <v>2</v>
       </c>
       <c r="G8" t="str">
-        <v>16.5%</v>
+        <v>85.7%</v>
       </c>
       <c r="H8" t="str">
         <v/>
       </c>
       <c r="I8" t="str">
-        <v>16203</v>
+        <v>29077</v>
       </c>
       <c r="J8" t="str">
-        <v>Tribunal de Oujda</v>
+        <v>Tribunal de Tanger</v>
       </c>
       <c r="K8" t="str">
         <v>Société à Responsabilité Limitée</v>
@@ -783,7 +783,7 @@
         <v>100 000 DHS</v>
       </c>
       <c r="M8" t="str">
-        <v>Ci3 n° 32 lot angad - Oujda-Angad</v>
+        <v>9, rue antaki, appt n° 1 - Tanger-Médina (AR)</v>
       </c>
       <c r="N8" t="str">
         <v/>
@@ -806,31 +806,31 @@
         <v>Not Found – Suggestion</v>
       </c>
       <c r="E9" t="str">
-        <v>STE FABRICATION ET DIVERS TRAVAUX (STE SOFADIT SARL)</v>
+        <v>SOFANOR</v>
       </c>
       <c r="F9">
         <v>3</v>
       </c>
       <c r="G9" t="str">
-        <v>25.0%</v>
+        <v>85.7%</v>
       </c>
       <c r="H9" t="str">
-        <v/>
+        <v>001653636000055</v>
       </c>
       <c r="I9" t="str">
-        <v>2389</v>
+        <v>45519</v>
       </c>
       <c r="J9" t="str">
-        <v>Tribunal de Errachidia</v>
+        <v>Tribunal de Fes</v>
       </c>
       <c r="K9" t="str">
-        <v>Société à Responsabilité Limitée</v>
+        <v>Société à Responsabilité Limitée à Associé Unique</v>
       </c>
       <c r="L9" t="str">
-        <v>100 000 DHS</v>
+        <v>10 000 DHS</v>
       </c>
       <c r="M9" t="str">
-        <v>01 rue 15 talat boutalamine - Errachidia</v>
+        <v>N° 3 bloc 5 bled el megzari sahrij gunaoua - Fès-Médina (AR)</v>
       </c>
       <c r="N9" t="str">
         <v/>
@@ -877,13 +877,13 @@
         <v>100 000 DHS</v>
       </c>
       <c r="M10" t="str">
-        <v/>
+        <v>Douar anounaadi chtouka ait baha - Chtouka- Ait Baha</v>
       </c>
       <c r="N10" t="str">
         <v/>
       </c>
       <c r="O10">
-        <v>2010</v>
+        <v>12162</v>
       </c>
     </row>
     <row r="11">
@@ -924,13 +924,13 @@
         <v>100 000 DHS</v>
       </c>
       <c r="M11" t="str">
-        <v/>
+        <v>Avenue mohamed v agdez - Zagora (M)</v>
       </c>
       <c r="N11" t="str">
         <v/>
       </c>
       <c r="O11">
-        <v>1485</v>
+        <v>7517</v>
       </c>
     </row>
     <row r="12">
@@ -971,13 +971,13 @@
         <v>100 000 DHS</v>
       </c>
       <c r="M12" t="str">
-        <v/>
+        <v>Douar elbuibate inchaden belfaa- massa-inchaden - Chtouka- Ait Baha</v>
       </c>
       <c r="N12" t="str">
         <v/>
       </c>
       <c r="O12">
-        <v>1580</v>
+        <v>1735</v>
       </c>
     </row>
     <row r="13">
@@ -1018,13 +1018,13 @@
         <v>100 000 DHS</v>
       </c>
       <c r="M13" t="str">
-        <v/>
+        <v>Bled rostal rue n°10 n°216 1er étage tabriquet - Tabriquet (AR)</v>
       </c>
       <c r="N13" t="str">
         <v/>
       </c>
       <c r="O13">
-        <v>1766</v>
+        <v>6781</v>
       </c>
     </row>
     <row r="14">
@@ -1065,13 +1065,13 @@
         <v>100 000 DHS</v>
       </c>
       <c r="M14" t="str">
-        <v/>
+        <v>Hay ouahda bloc 1 gpe 7 no 9 - Sidi Yahya El Gharb (M)</v>
       </c>
       <c r="N14" t="str">
         <v/>
       </c>
       <c r="O14">
-        <v>1703</v>
+        <v>17484</v>
       </c>
     </row>
     <row r="15">
@@ -1085,25 +1085,25 @@
         <v>MARRAKECH</v>
       </c>
       <c r="D15" t="str">
-        <v>Not Found – Suggestion</v>
+        <v>Found</v>
       </c>
       <c r="E15" t="str">
-        <v>RIDS</v>
-      </c>
-      <c r="F15">
-        <v>1</v>
+        <v>HOLIDAY.RIDS</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
       </c>
       <c r="G15" t="str">
-        <v>25.0%</v>
+        <v>100.0%</v>
       </c>
       <c r="H15" t="str">
-        <v>001910899000027</v>
+        <v>003028124000012</v>
       </c>
       <c r="I15" t="str">
-        <v>22191</v>
+        <v>125331</v>
       </c>
       <c r="J15" t="str">
-        <v>Tribunal de Tetouan</v>
+        <v>Tribunal de Marrakech</v>
       </c>
       <c r="K15" t="str">
         <v>Société à Responsabilité Limitée à Associé Unique</v>
@@ -1112,124 +1112,124 @@
         <v>100 000 DHS</v>
       </c>
       <c r="M15" t="str">
-        <v>Av . mly . lhassan ben al mahdi n°190 -93000 - Tetouan (M)</v>
+        <v>Quartier industriel sidi ghanem n°206 2eme etage bureau n°3 - Marrakech-Médina (AR)</v>
       </c>
       <c r="N15" t="str">
         <v/>
       </c>
       <c r="O15">
-        <v>3624</v>
+        <v>43699</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>1735673</v>
+        <v>1735883</v>
       </c>
       <c r="B16" t="str">
-        <v>STE HOLIDAY RIDS</v>
+        <v>STE TRANSPORT FARHANA</v>
       </c>
       <c r="C16" t="str">
-        <v>MARRAKECH</v>
+        <v>OUARZAZATE</v>
       </c>
       <c r="D16" t="str">
-        <v>Not Found – Suggestion</v>
+        <v>Found</v>
       </c>
       <c r="E16" t="str">
-        <v>GREAT HOLIDAY RESIDENCE</v>
-      </c>
-      <c r="F16">
-        <v>2</v>
+        <v>SOCIETE TRANSPORT FARHANA</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
       </c>
       <c r="G16" t="str">
-        <v>56.5%</v>
+        <v>100.0%</v>
       </c>
       <c r="H16" t="str">
-        <v>003052602000064</v>
+        <v>001858048000037</v>
       </c>
       <c r="I16" t="str">
-        <v>51167</v>
+        <v>1765</v>
       </c>
       <c r="J16" t="str">
-        <v>Tribunal de Agadir</v>
+        <v>Tribunal de Ouarzazate</v>
       </c>
       <c r="K16" t="str">
-        <v>Société à Responsabilité Limitée à Associé Unique</v>
+        <v>Société à Responsabilité Limitée</v>
       </c>
       <c r="L16" t="str">
-        <v>5 100 000 DHS</v>
+        <v>100 000 DHS</v>
       </c>
       <c r="M16" t="str">
-        <v>Residence khalij ennakhil lotissement g7 founti - Agadir (M)</v>
+        <v>N23 rue de marche - Ouarzazate</v>
       </c>
       <c r="N16" t="str">
         <v/>
       </c>
-      <c r="O16" t="str">
-        <v/>
+      <c r="O16">
+        <v>12834</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>1735673</v>
+        <v>1736382</v>
       </c>
       <c r="B17" t="str">
-        <v>STE HOLIDAY RIDS</v>
+        <v>CHAMA LUXURY SARL AU</v>
       </c>
       <c r="C17" t="str">
         <v>MARRAKECH</v>
       </c>
       <c r="D17" t="str">
-        <v>Not Found – Suggestion</v>
+        <v>Found</v>
       </c>
       <c r="E17" t="str">
-        <v>MOON HOLIDAY</v>
-      </c>
-      <c r="F17">
-        <v>3</v>
+        <v>CHAMA LUXURY</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
       </c>
       <c r="G17" t="str">
-        <v>43.8%</v>
+        <v>100.0%</v>
       </c>
       <c r="H17" t="str">
-        <v/>
+        <v>001858306000055</v>
       </c>
       <c r="I17" t="str">
-        <v>134693</v>
+        <v>79289</v>
       </c>
       <c r="J17" t="str">
-        <v>Tribunal de Casablanca</v>
+        <v>Tribunal de Marrakech</v>
       </c>
       <c r="K17" t="str">
-        <v>Société à Responsabilité Limitée</v>
+        <v>Société à Responsabilité Limitée à Associé Unique</v>
       </c>
       <c r="L17" t="str">
-        <v>1 000 000 DHS</v>
+        <v>100 000 DHS</v>
       </c>
       <c r="M17" t="str">
-        <v>Rue n1 jabel el aroui villa n° 11 hay essalam cil - Casablanca</v>
+        <v>N°123 lot yassmine 2 izdihar - Marrakech-Médina (AR)</v>
       </c>
       <c r="N17" t="str">
         <v/>
       </c>
-      <c r="O17" t="str">
-        <v/>
+      <c r="O17">
+        <v>18037</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>1735883</v>
+        <v>1736759</v>
       </c>
       <c r="B18" t="str">
-        <v>STE TRANSPORT FARHANA</v>
+        <v>STE TRANSPORT TOURISTIQUE DISTRACTION SARL</v>
       </c>
       <c r="C18" t="str">
-        <v>OUARZAZATE</v>
+        <v>NADOR</v>
       </c>
       <c r="D18" t="str">
         <v>Found</v>
       </c>
       <c r="E18" t="str">
-        <v>SOCIETE TRANSPORT FARHANA</v>
+        <v>TRANSPORT TOURISTIQUE DISTRACTION</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -1238,210 +1238,210 @@
         <v>100.0%</v>
       </c>
       <c r="H18" t="str">
-        <v>001858048000037</v>
+        <v>001823623000058</v>
       </c>
       <c r="I18" t="str">
-        <v>1765</v>
+        <v>15845</v>
       </c>
       <c r="J18" t="str">
-        <v>Tribunal de Ouarzazate</v>
+        <v>Tribunal de Nador</v>
       </c>
       <c r="K18" t="str">
         <v>Société à Responsabilité Limitée</v>
       </c>
       <c r="L18" t="str">
-        <v>100 000 DHS</v>
+        <v>160 000 DHS</v>
       </c>
       <c r="M18" t="str">
-        <v/>
+        <v>Beni enzar centre - Nador (M)</v>
       </c>
       <c r="N18" t="str">
         <v/>
       </c>
       <c r="O18">
-        <v>1763</v>
+        <v>17656</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>1736382</v>
+        <v>1738023</v>
       </c>
       <c r="B19" t="str">
-        <v>CHAMA LUXURY SARL AU</v>
+        <v>STE MONY SPEED</v>
       </c>
       <c r="C19" t="str">
-        <v>MARRAKECH</v>
+        <v>KHOURIBGA</v>
       </c>
       <c r="D19" t="str">
-        <v>Found</v>
+        <v>Not Found – Suggestion</v>
       </c>
       <c r="E19" t="str">
-        <v>CHAMA LUXURY</v>
-      </c>
-      <c r="F19" t="str">
-        <v/>
+        <v>MOTSPEED</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
       </c>
       <c r="G19" t="str">
-        <v>80.0%</v>
+        <v>77.8%</v>
       </c>
       <c r="H19" t="str">
-        <v>001858306000055</v>
+        <v>000063161000010</v>
       </c>
       <c r="I19" t="str">
-        <v>79289</v>
+        <v>53969</v>
       </c>
       <c r="J19" t="str">
-        <v>Tribunal de Marrakech</v>
+        <v>Tribunal de Tanger</v>
       </c>
       <c r="K19" t="str">
-        <v>Société à Responsabilité Limitée à Associé Unique</v>
+        <v>Société à Responsabilité Limitée</v>
       </c>
       <c r="L19" t="str">
         <v>100 000 DHS</v>
       </c>
       <c r="M19" t="str">
-        <v/>
+        <v>Lot al amal 1 rue 4 n° 52 - Tanger-Médina (AR)</v>
       </c>
       <c r="N19" t="str">
         <v/>
       </c>
       <c r="O19">
-        <v>1656</v>
+        <v>25636</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>1736759</v>
+        <v>1712758</v>
       </c>
       <c r="B20" t="str">
-        <v>STE TRANSPORT TOURISTIQUE DISTRACTION SARL</v>
+        <v>CHAME CAR</v>
       </c>
       <c r="C20" t="str">
-        <v>NADOR</v>
+        <v>MARRAKECH</v>
       </c>
       <c r="D20" t="str">
-        <v>Found</v>
+        <v>Not Found – Suggestion</v>
       </c>
       <c r="E20" t="str">
-        <v>TRANSPORT TOURISTIQUE DISTRACTION</v>
-      </c>
-      <c r="F20" t="str">
-        <v/>
+        <v>CHAMAR (CHAMAR)</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
       </c>
       <c r="G20" t="str">
-        <v>100.0%</v>
+        <v>61.5%</v>
       </c>
       <c r="H20" t="str">
-        <v>001823623000058</v>
+        <v/>
       </c>
       <c r="I20" t="str">
-        <v>15845</v>
+        <v>10446</v>
       </c>
       <c r="J20" t="str">
-        <v>Tribunal de Nador</v>
+        <v>Tribunal de Fes</v>
       </c>
       <c r="K20" t="str">
-        <v>Société à Responsabilité Limitée</v>
+        <v>Société Anonyme</v>
       </c>
       <c r="L20" t="str">
-        <v>160 000 DHS</v>
+        <v>1 500 000 DHS</v>
       </c>
       <c r="M20" t="str">
-        <v/>
+        <v>Rue d'espagne - Fès</v>
       </c>
       <c r="N20" t="str">
         <v/>
       </c>
       <c r="O20">
-        <v>2693</v>
+        <v>42476</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>1738023</v>
+        <v>1712758</v>
       </c>
       <c r="B21" t="str">
-        <v>STE MONY SPEED</v>
+        <v>CHAME CAR</v>
       </c>
       <c r="C21" t="str">
-        <v>KHOURIBGA</v>
+        <v>MARRAKECH</v>
       </c>
       <c r="D21" t="str">
         <v>Not Found – Suggestion</v>
       </c>
       <c r="E21" t="str">
-        <v>MONY SPEED CAR</v>
+        <v>CAMECAS</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21" t="str">
-        <v>42.9%</v>
+        <v>75.0%</v>
       </c>
       <c r="H21" t="str">
-        <v>002901863000091</v>
+        <v/>
       </c>
       <c r="I21" t="str">
-        <v>7231</v>
+        <v>7981</v>
       </c>
       <c r="J21" t="str">
-        <v>Tribunal de Khouribga</v>
+        <v>Tribunal de Eljadida</v>
       </c>
       <c r="K21" t="str">
         <v>Société à Responsabilité Limitée à Associé Unique</v>
       </c>
       <c r="L21" t="str">
-        <v>500 000 DHS</v>
+        <v>100 000 DHS</v>
       </c>
       <c r="M21" t="str">
-        <v>9 lotissement el wahidi etg 1 apt 1 - Khouribga (M)</v>
+        <v>8 rue iraq - El-Jadida (M)</v>
       </c>
       <c r="N21" t="str">
         <v/>
       </c>
-      <c r="O21">
-        <v>4017</v>
+      <c r="O21" t="str">
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>1738023</v>
+        <v>1712758</v>
       </c>
       <c r="B22" t="str">
-        <v>STE MONY SPEED</v>
+        <v>CHAME CAR</v>
       </c>
       <c r="C22" t="str">
-        <v>KHOURIBGA</v>
+        <v>MARRAKECH</v>
       </c>
       <c r="D22" t="str">
         <v>Not Found – Suggestion</v>
       </c>
       <c r="E22" t="str">
-        <v>TIGHIRT MONY CASH</v>
+        <v>CHAMEC</v>
       </c>
       <c r="F22">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G22" t="str">
-        <v>29.4%</v>
+        <v>75.0%</v>
       </c>
       <c r="H22" t="str">
-        <v>001389919000032</v>
+        <v>000092693000083</v>
       </c>
       <c r="I22" t="str">
-        <v>19683</v>
+        <v>131959</v>
       </c>
       <c r="J22" t="str">
-        <v>Tribunal de Inzegane</v>
+        <v>Tribunal de Casablanca</v>
       </c>
       <c r="K22" t="str">
-        <v>Société à Responsabilité Limitée</v>
+        <v>Société à Responsabilité Limitée à Associé Unique</v>
       </c>
       <c r="L22" t="str">
         <v>100 000 DHS</v>
       </c>
       <c r="M22" t="str">
-        <v>Rue 3206 n32 hay igui ferden - Dcheira El Jihadia (M)</v>
+        <v>19, rue haj omar riffi - Casablanca</v>
       </c>
       <c r="N22" t="str">
         <v/>
@@ -1452,289 +1452,101 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>1738023</v>
+        <v>1713261</v>
       </c>
       <c r="B23" t="str">
-        <v>STE MONY SPEED</v>
+        <v>STE INRZAF TRANS</v>
       </c>
       <c r="C23" t="str">
-        <v>KHOURIBGA</v>
+        <v>OUARZAZATE</v>
       </c>
       <c r="D23" t="str">
-        <v>Not Found – Suggestion</v>
+        <v>Found</v>
       </c>
       <c r="E23" t="str">
-        <v>STE SPEED MIXLUB</v>
-      </c>
-      <c r="F23">
-        <v>3</v>
+        <v>INRZAF TRANS</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
       </c>
       <c r="G23" t="str">
-        <v>31.3%</v>
+        <v>100.0%</v>
       </c>
       <c r="H23" t="str">
-        <v>002129785000024</v>
+        <v>003016426000026</v>
       </c>
       <c r="I23" t="str">
-        <v>56595</v>
+        <v>11867</v>
       </c>
       <c r="J23" t="str">
-        <v>Tribunal de Fes</v>
+        <v>Tribunal de Ouarzazate</v>
       </c>
       <c r="K23" t="str">
         <v>Société à Responsabilité Limitée</v>
       </c>
       <c r="L23" t="str">
-        <v>430 000 DHS</v>
+        <v>100 000 DHS</v>
       </c>
       <c r="M23" t="str">
-        <v>N°103 lots jnane zaytoune cooperative mahdia bensouda - Fès-Médina (AR)</v>
+        <v>Dr islday ighrem nougdal - Ighrem N'Ougdal</v>
       </c>
       <c r="N23" t="str">
         <v/>
       </c>
-      <c r="O23" t="str">
-        <v/>
+      <c r="O23">
+        <v>17889</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>1712758</v>
+        <v>1713823</v>
       </c>
       <c r="B24" t="str">
-        <v>CHAME CAR</v>
+        <v>STE FOURAGE TIZI</v>
       </c>
       <c r="C24" t="str">
-        <v>MARRAKECH</v>
+        <v>DRIOUCH</v>
       </c>
       <c r="D24" t="str">
-        <v>Not Found – Suggestion</v>
+        <v>Found</v>
       </c>
       <c r="E24" t="str">
-        <v>MY CAR (MY CAR)</v>
-      </c>
-      <c r="F24">
-        <v>1</v>
+        <v>FOURAGE TIZI</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
       </c>
       <c r="G24" t="str">
-        <v>40.0%</v>
+        <v>100.0%</v>
       </c>
       <c r="H24" t="str">
-        <v>001540767000069</v>
+        <v>002527630000086</v>
       </c>
       <c r="I24" t="str">
-        <v>42715</v>
+        <v>105</v>
       </c>
       <c r="J24" t="str">
-        <v>Tribunal de Casablanca</v>
+        <v>Tribunal de Driouch</v>
       </c>
       <c r="K24" t="str">
         <v>Société à Responsabilité Limitée</v>
       </c>
       <c r="L24" t="str">
-        <v>570 000 DHS</v>
+        <v>2 100 000 DHS</v>
       </c>
       <c r="M24" t="str">
-        <v>Bd mohamed vi -ex route de mediouna n 507 a 519 el fida - Al-Fida (AR)</v>
+        <v>Hay saada 02 driouch - Driouch</v>
       </c>
       <c r="N24" t="str">
         <v/>
       </c>
       <c r="O24">
-        <v>3365</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>1712758</v>
-      </c>
-      <c r="B25" t="str">
-        <v>CHAME CAR</v>
-      </c>
-      <c r="C25" t="str">
-        <v>MARRAKECH</v>
-      </c>
-      <c r="D25" t="str">
-        <v>Not Found – Suggestion</v>
-      </c>
-      <c r="E25" t="str">
-        <v>RES@CAR (RES@CAR)</v>
-      </c>
-      <c r="F25">
-        <v>2</v>
-      </c>
-      <c r="G25" t="str">
-        <v>29.4%</v>
-      </c>
-      <c r="H25" t="str">
-        <v>000222720000075</v>
-      </c>
-      <c r="I25" t="str">
-        <v>9807</v>
-      </c>
-      <c r="J25" t="str">
-        <v>Tribunal de Mohammedia</v>
-      </c>
-      <c r="K25" t="str">
-        <v>Société à Responsabilité Limitée</v>
-      </c>
-      <c r="L25" t="str">
-        <v>10 000 DHS</v>
-      </c>
-      <c r="M25" t="str">
-        <v>Lotissement wafaa rdc n 179 - Mohammedia (M)</v>
-      </c>
-      <c r="N25" t="str">
-        <v/>
-      </c>
-      <c r="O25" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>1712758</v>
-      </c>
-      <c r="B26" t="str">
-        <v>CHAME CAR</v>
-      </c>
-      <c r="C26" t="str">
-        <v>MARRAKECH</v>
-      </c>
-      <c r="D26" t="str">
-        <v>Not Found – Suggestion</v>
-      </c>
-      <c r="E26" t="str">
-        <v>ZEIN CHAME</v>
-      </c>
-      <c r="F26">
-        <v>3</v>
-      </c>
-      <c r="G26" t="str">
-        <v>20.0%</v>
-      </c>
-      <c r="H26" t="str">
-        <v>000080916000096</v>
-      </c>
-      <c r="I26" t="str">
-        <v>43499</v>
-      </c>
-      <c r="J26" t="str">
-        <v>Tribunal de Marrakech</v>
-      </c>
-      <c r="K26" t="str">
-        <v>Société à Responsabilité Limitée</v>
-      </c>
-      <c r="L26" t="str">
-        <v>450 000 DHS</v>
-      </c>
-      <c r="M26" t="str">
-        <v>55 res errahma av abdelkrim el khattabi - Gueliz (AR)</v>
-      </c>
-      <c r="N26" t="str">
-        <v/>
-      </c>
-      <c r="O26" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>1713261</v>
-      </c>
-      <c r="B27" t="str">
-        <v>STE INRZAF TRANS</v>
-      </c>
-      <c r="C27" t="str">
-        <v>OUARZAZATE</v>
-      </c>
-      <c r="D27" t="str">
-        <v>Found</v>
-      </c>
-      <c r="E27" t="str">
-        <v>INRZAF TRANS</v>
-      </c>
-      <c r="F27" t="str">
-        <v/>
-      </c>
-      <c r="G27" t="str">
-        <v>100.0%</v>
-      </c>
-      <c r="H27" t="str">
-        <v>003016426000026</v>
-      </c>
-      <c r="I27" t="str">
-        <v>11867</v>
-      </c>
-      <c r="J27" t="str">
-        <v>Tribunal de Ouarzazate</v>
-      </c>
-      <c r="K27" t="str">
-        <v>Société à Responsabilité Limitée</v>
-      </c>
-      <c r="L27" t="str">
-        <v>100 000 DHS</v>
-      </c>
-      <c r="M27" t="str">
-        <v/>
-      </c>
-      <c r="N27" t="str">
-        <v/>
-      </c>
-      <c r="O27">
-        <v>1838</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>1713823</v>
-      </c>
-      <c r="B28" t="str">
-        <v>STE FOURAGE TIZI</v>
-      </c>
-      <c r="C28" t="str">
-        <v>DRIOUCH</v>
-      </c>
-      <c r="D28" t="str">
-        <v>Found</v>
-      </c>
-      <c r="E28" t="str">
-        <v>FOURAGE TIZI</v>
-      </c>
-      <c r="F28" t="str">
-        <v/>
-      </c>
-      <c r="G28" t="str">
-        <v>100.0%</v>
-      </c>
-      <c r="H28" t="str">
-        <v>002527630000086</v>
-      </c>
-      <c r="I28" t="str">
-        <v>105</v>
-      </c>
-      <c r="J28" t="str">
-        <v>Tribunal de Driouch</v>
-      </c>
-      <c r="K28" t="str">
-        <v>Société à Responsabilité Limitée</v>
-      </c>
-      <c r="L28" t="str">
-        <v>2 100 000 DHS</v>
-      </c>
-      <c r="M28" t="str">
-        <v/>
-      </c>
-      <c r="N28" t="str">
-        <v/>
-      </c>
-      <c r="O28">
-        <v>1624</v>
+        <v>1691</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>